<commit_message>
se ajusta barra de progreso, se ajusta, interactividad con la app mientras esta en ejecucion
</commit_message>
<xml_diff>
--- a/Correccion_nombres_base_subgerentes.xlsx
+++ b/Correccion_nombres_base_subgerentes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,18 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>GISELA ZAMORA DIAZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>JOSE MARTINEZZ</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>JOSE MARTINEZ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se agregan validaciones, se agrega pestaña para los cajeros que no se encontraron en base seguro actualiza
</commit_message>
<xml_diff>
--- a/Correccion_nombres_base_subgerentes.xlsx
+++ b/Correccion_nombres_base_subgerentes.xlsx
@@ -1,40 +1,111 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
   <workbookPr/>
-  <workbookProtection/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{69343BB2-1EA6-4656-A404-1D7C9944479C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Subgerentes" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>Base Subgerentes</t>
+  </si>
+  <si>
+    <t>NOMBRE ERRONEO</t>
+  </si>
+  <si>
+    <t>NOMBRE CORRECTO A CAMBIAR</t>
+  </si>
+  <si>
+    <t>GISELLA ZAMORA DIAZ</t>
+  </si>
+  <si>
+    <t>GISELA ZAMORA DIAZ</t>
+  </si>
+  <si>
+    <t>JOSE MARTINEZZ</t>
+  </si>
+  <si>
+    <t>JOSE MARTINEZ</t>
+  </si>
+  <si>
+    <t>CEDULA</t>
+  </si>
+  <si>
+    <t>USUARIO WINDOWS</t>
+  </si>
+  <si>
+    <t>INICIALES</t>
+  </si>
+  <si>
+    <t>COLABORADOR</t>
+  </si>
+  <si>
+    <t>CARGO</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +113,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,58 +444,81 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Base Subgerentes</t>
-        </is>
-      </c>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NOMBRE ERRONEO</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NOMBRE CORRECTO A CAMBIAR</t>
-        </is>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>GISELLA ZAMORA DIAZ</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GISELA ZAMORA DIAZ</t>
-        </is>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>JOSE MARTINEZZ</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>JOSE MARTINEZ</t>
-        </is>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1368654D-EF86-4BEF-BF25-7F31B26FDB17}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="28.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="2" customFormat="1">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
se sube archivo excel de pruebas para validar el error de inconcistencias de valores de prima para subgerente
</commit_message>
<xml_diff>
--- a/Correccion_nombres_base_subgerentes.xlsx
+++ b/Correccion_nombres_base_subgerentes.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69343BB2-1EA6-4656-A404-1D7C9944479C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PedrazaJh\Proyectos\Banco w\2026_INSENTIVOS_BANCO_W\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{704701C5-1D02-4D30-952F-E609150D521A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -32,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Base Subgerentes</t>
   </si>
@@ -68,13 +73,64 @@
   </si>
   <si>
     <t>CARGO</t>
+  </si>
+  <si>
+    <t>BCASTILLO</t>
+  </si>
+  <si>
+    <t>DBN</t>
+  </si>
+  <si>
+    <t>DMJIMENEZ</t>
+  </si>
+  <si>
+    <t>GDH</t>
+  </si>
+  <si>
+    <t>EPALACIOS</t>
+  </si>
+  <si>
+    <t>IVW</t>
+  </si>
+  <si>
+    <t>JESTACIO</t>
+  </si>
+  <si>
+    <t>RDO</t>
+  </si>
+  <si>
+    <t>ESTACIO ARDILA JULIO CESAR</t>
+  </si>
+  <si>
+    <t>VDRADA</t>
+  </si>
+  <si>
+    <t>MSU</t>
+  </si>
+  <si>
+    <t>AUXILIAR OPERATIVO</t>
+  </si>
+  <si>
+    <t>BELLA LIVIS CASTILLO GIL</t>
+  </si>
+  <si>
+    <t>DIANA MAYERLY JIMENEZ MARIN</t>
+  </si>
+  <si>
+    <t>EVANS PALACIOS ANGULO</t>
+  </si>
+  <si>
+    <t>VALENTINA DRADA COBALEDA</t>
+  </si>
+  <si>
+    <t>CAJERO(A) PRINCIPAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,16 +188,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -446,19 +511,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="B1" s="3"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -466,7 +531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -474,7 +539,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -492,30 +557,114 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1368654D-EF86-4BEF-BF25-7F31B26FDB17}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="28.42578125" customWidth="1"/>
+    <col min="1" max="1" width="15.54296875" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.90625" customWidth="1"/>
+    <col min="4" max="4" width="41.36328125" customWidth="1"/>
+    <col min="5" max="5" width="24.1796875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="5" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="4">
+        <v>1065002794</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>1088256473</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>1111793303</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>1087185918</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>1007609499</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>